<commit_message>
Realizar coleta das colunas do SILT
</commit_message>
<xml_diff>
--- a/dados/sonda_cobertura_dou.xlsx
+++ b/dados/sonda_cobertura_dou.xlsx
@@ -1135,13 +1135,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5E14363F-E532-463C-B3C5-40B2F4A6755D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{35519F97-CFC7-4A9D-B1FE-DD9BA984B2E8}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AFDD29A3-9261-4599-98B4-187308C7D31A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7AA20D3A-4294-4085-AAF1-9B7BC5530528}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F56A7893-ABD5-4751-A14F-668221C9C4DD}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{166836D7-37CB-46CA-A707-0E0CB84D534B}"/>
 </file>
</xml_diff>